<commit_message>
Add travel times, a table of all routes and a scorecard per carrier to the page
Travel time rebuilds the paper's travel model (graph.TransitGraph) in the
browser and shows the estimated minutes by bus from any stop; from 15 stops it
gives the same counts per 15-minute band as the Python model. The table of all
201 routes and the table of the 39 carriers sort on any column and filter on
their text; carrier names that differ only in spelling are counted once, and a
carrier's row draws its routes on the map. The checklist gains a Carriers sheet.
</commit_message>
<xml_diff>
--- a/site/checklist.xlsx
+++ b/site/checklist.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Near-duplicate routes" sheetId="4" r:id="rId4"/>
     <sheet name="Corridors" sheetId="5" r:id="rId5"/>
     <sheet name="Close stops" sheetId="6" r:id="rId6"/>
-    <sheet name="Routes" sheetId="7" r:id="rId7"/>
+    <sheet name="Carriers" sheetId="7" r:id="rId7"/>
+    <sheet name="Routes" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data issues'!$A$1:$D$41</definedName>
@@ -19,7 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Near-duplicate routes'!$A$1:$H$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Corridors'!$A$1:$H$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Close stops'!$A$1:$D$352</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Routes'!$A$1:$R$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Carriers'!$A$1:$N$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Routes'!$A$1:$R$202</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -172,19 +174,26 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="6">
         <is>
-          <t>Routes: the measured figures for every route. Residents are counted within 400 m; boardings are published for BakuBus routes only.</t>
+          <t>Carriers: the routes each carrier runs and what they measure. AYNA plans the routes, so these figures describe the routes, not how well a carrier runs them. Names that differ only in spelling are counted once.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="6">
         <is>
-          <t>Page: https://ismatsamadov.github.io/route_efficiency/</t>
+          <t>Routes: the measured figures for every route. Residents are counted within 400 m; boardings are published for BakuBus routes only.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="6">
+        <is>
+          <t>Page: https://ismatsamadov.github.io/route_efficiency/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="6">
         <is>
           <t>Code, data and paper: https://github.com/ismatsamadov/route_efficiency</t>
         </is>
@@ -24921,6 +24930,1762 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>Carrier</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>Also spelled</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Routes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>Route numbers</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>One-way km</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>Direct routes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>Median path / straight line</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>Detours</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>Detour extra km</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>Routes mostly inside another route</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>… inside another carrier's route</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>Close stops served</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>Residents only one of its routes reaches</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t>Weekday boardings (BakuBus, 2026-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="6">
+        <is>
+          <t>BakuBus MMC</t>
+        </is>
+      </c>
+      <c r="C2" s="2">
+        <v>55</v>
+      </c>
+      <c r="D2" t="inlineStr" s="6">
+        <is>
+          <t>1 E1 H1 2 3 4 5 6 7A 7B M8 10 11 13 14 17 20 21 24 30 32 33 35 44 46 57 60 62 72 88 88A 108A 120 120E 121E 125 130 139 140 140E 141E 147 149 150 150E 163 172 189 205 211 217 503 508 594 595</t>
+        </is>
+      </c>
+      <c r="E2" s="3">
+        <v>1229.963</v>
+      </c>
+      <c r="F2" s="2">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4">
+        <v>1.7522</v>
+      </c>
+      <c r="H2" s="2">
+        <v>92</v>
+      </c>
+      <c r="I2" s="3">
+        <v>300.7337</v>
+      </c>
+      <c r="J2" s="2">
+        <v>2</v>
+      </c>
+      <c r="K2" s="2">
+        <v>2</v>
+      </c>
+      <c r="L2" s="2">
+        <v>149</v>
+      </c>
+      <c r="M2" s="2">
+        <v>71117.143</v>
+      </c>
+      <c r="N2" s="2">
+        <v>672788.8443</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="6">
+        <is>
+          <t>Çinar-Trans MMC</t>
+        </is>
+      </c>
+      <c r="C3" s="2">
+        <v>19</v>
+      </c>
+      <c r="D3" t="inlineStr" s="6">
+        <is>
+          <t>40 66 81 91 100 108B 133 145 160 160A 165 173A 173B 177 179 185 190 202 203</t>
+        </is>
+      </c>
+      <c r="E3" s="3">
+        <v>302.3866</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4">
+        <v>1.6461</v>
+      </c>
+      <c r="H3" s="2">
+        <v>21</v>
+      </c>
+      <c r="I3" s="3">
+        <v>73.4558</v>
+      </c>
+      <c r="J3" s="2">
+        <v>5</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>54</v>
+      </c>
+      <c r="M3" s="2">
+        <v>23551.7143</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="6">
+        <is>
+          <t>Xaliq Faiqoğlu MMC</t>
+        </is>
+      </c>
+      <c r="C4" s="2">
+        <v>18</v>
+      </c>
+      <c r="D4" t="inlineStr" s="6">
+        <is>
+          <t>9 18 37 41 45 52 61 65 79 85 96 114A 114B 119 135 170 199 592</t>
+        </is>
+      </c>
+      <c r="E4" s="3">
+        <v>252.977</v>
+      </c>
+      <c r="F4" s="2">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1.85275</v>
+      </c>
+      <c r="H4" s="2">
+        <v>19</v>
+      </c>
+      <c r="I4" s="3">
+        <v>51.975</v>
+      </c>
+      <c r="J4" s="2">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>32</v>
+      </c>
+      <c r="M4" s="2">
+        <v>11666.8571</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="6">
+        <is>
+          <t>BUS TRANS MMC</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr" s="6">
+        <is>
+          <t>51 102 104 106 112 155 157 169 183 206</t>
+        </is>
+      </c>
+      <c r="E5" s="3">
+        <v>171.58520000000001</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>2.4077</v>
+      </c>
+      <c r="H5" s="2">
+        <v>18</v>
+      </c>
+      <c r="I5" s="3">
+        <v>85.4945</v>
+      </c>
+      <c r="J5" s="2">
+        <v>2</v>
+      </c>
+      <c r="K5" s="2">
+        <v>2</v>
+      </c>
+      <c r="L5" s="2">
+        <v>45</v>
+      </c>
+      <c r="M5" s="2">
+        <v>17940.2856</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="6">
+        <is>
+          <t>BMHMMC</t>
+        </is>
+      </c>
+      <c r="C6" s="2">
+        <v>9</v>
+      </c>
+      <c r="D6" t="inlineStr" s="6">
+        <is>
+          <t>111 120A 126 140A 164 174 176 194 195</t>
+        </is>
+      </c>
+      <c r="E6" s="3">
+        <v>215.2094</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1.6704</v>
+      </c>
+      <c r="H6" s="2">
+        <v>9</v>
+      </c>
+      <c r="I6" s="3">
+        <v>42.5965</v>
+      </c>
+      <c r="J6" s="2">
+        <v>2</v>
+      </c>
+      <c r="K6" s="2">
+        <v>2</v>
+      </c>
+      <c r="L6" s="2">
+        <v>20</v>
+      </c>
+      <c r="M6" s="2">
+        <v>17689.7142</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="6">
+        <is>
+          <t>6 Dost MMC</t>
+        </is>
+      </c>
+      <c r="C7" s="2">
+        <v>7</v>
+      </c>
+      <c r="D7" t="inlineStr" s="6">
+        <is>
+          <t>101 143 146 162 180 182 213</t>
+        </is>
+      </c>
+      <c r="E7" s="3">
+        <v>115.7743</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="4">
+        <v>1.7857</v>
+      </c>
+      <c r="H7" s="2">
+        <v>5</v>
+      </c>
+      <c r="I7" s="3">
+        <v>21.9948</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <v>7</v>
+      </c>
+      <c r="M7" s="2">
+        <v>11101.2857</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="6">
+        <is>
+          <t>F.RÖVŞƏN İSTEHSALAT MÜƏSSİSƏSİ</t>
+        </is>
+      </c>
+      <c r="C8" s="2">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr" s="6">
+        <is>
+          <t>123 506 515 522 523 535 596</t>
+        </is>
+      </c>
+      <c r="E8" s="3">
+        <v>151.2461</v>
+      </c>
+      <c r="F8" s="2">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4">
+        <v>1.554</v>
+      </c>
+      <c r="H8" s="2">
+        <v>6</v>
+      </c>
+      <c r="I8" s="3">
+        <v>17.4454</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>34</v>
+      </c>
+      <c r="M8" s="2">
+        <v>21739.142799999998</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="6">
+        <is>
+          <t>General - Auto - Company firması</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="6">
+        <is>
+          <t>General-Auto-Company firması</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <v>7</v>
+      </c>
+      <c r="D9" t="inlineStr" s="6">
+        <is>
+          <t>15 38 64 131 166 184 216</t>
+        </is>
+      </c>
+      <c r="E9" s="3">
+        <v>111.69290000000001</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1.9523</v>
+      </c>
+      <c r="H9" s="2">
+        <v>11</v>
+      </c>
+      <c r="I9" s="3">
+        <v>36.6816</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <v>35</v>
+      </c>
+      <c r="M9" s="2">
+        <v>5250.4286</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="6">
+        <is>
+          <t>Kənan-2000 şirkəti</t>
+        </is>
+      </c>
+      <c r="C10" s="2">
+        <v>6</v>
+      </c>
+      <c r="D10" t="inlineStr" s="6">
+        <is>
+          <t>22 70 118A 142 191 204</t>
+        </is>
+      </c>
+      <c r="E10" s="3">
+        <v>85.3661</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>1.7608000000000001</v>
+      </c>
+      <c r="H10" s="2">
+        <v>9</v>
+      </c>
+      <c r="I10" s="3">
+        <v>35.2292</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2">
+        <v>27</v>
+      </c>
+      <c r="M10" s="2">
+        <v>15492.5714</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="6">
+        <is>
+          <t>SAHİL MMC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="6">
+        <is>
+          <t>Sahil MMC</t>
+        </is>
+      </c>
+      <c r="C11" s="2">
+        <v>6</v>
+      </c>
+      <c r="D11" t="inlineStr" s="6">
+        <is>
+          <t>159 505 517 531 533 557</t>
+        </is>
+      </c>
+      <c r="E11" s="3">
+        <v>131.8622</v>
+      </c>
+      <c r="F11" s="2">
+        <v>2</v>
+      </c>
+      <c r="G11" s="4">
+        <v>1.59175</v>
+      </c>
+      <c r="H11" s="2">
+        <v>6</v>
+      </c>
+      <c r="I11" s="3">
+        <v>22.2762</v>
+      </c>
+      <c r="J11" s="2">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2">
+        <v>13</v>
+      </c>
+      <c r="M11" s="2">
+        <v>14028.2857</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="6">
+        <is>
+          <t>Vətən.Az-Trans MMC</t>
+        </is>
+      </c>
+      <c r="C12" s="2">
+        <v>6</v>
+      </c>
+      <c r="D12" t="inlineStr" s="6">
+        <is>
+          <t>12 36 50 210 212 215</t>
+        </is>
+      </c>
+      <c r="E12" s="3">
+        <v>76.0994</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>1.8514499999999998</v>
+      </c>
+      <c r="H12" s="2">
+        <v>12</v>
+      </c>
+      <c r="I12" s="3">
+        <v>37.8496</v>
+      </c>
+      <c r="J12" s="2">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
+        <v>17</v>
+      </c>
+      <c r="M12" s="2">
+        <v>5889.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="6">
+        <is>
+          <t>MENLOQQ MMC</t>
+        </is>
+      </c>
+      <c r="C13" s="2">
+        <v>5</v>
+      </c>
+      <c r="D13" t="inlineStr" s="6">
+        <is>
+          <t>29 67 71 83 103</t>
+        </is>
+      </c>
+      <c r="E13" s="3">
+        <v>78.4509</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>2.098</v>
+      </c>
+      <c r="H13" s="2">
+        <v>11</v>
+      </c>
+      <c r="I13" s="3">
+        <v>25.9649</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>37</v>
+      </c>
+      <c r="M13" s="2">
+        <v>19421.5714</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="6">
+        <is>
+          <t>Ayşən LTD MMC</t>
+        </is>
+      </c>
+      <c r="C14" s="2">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr" s="6">
+        <is>
+          <t>107 168 186 214</t>
+        </is>
+      </c>
+      <c r="E14" s="3">
+        <v>108.7795</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>1.7289</v>
+      </c>
+      <c r="H14" s="2">
+        <v>8</v>
+      </c>
+      <c r="I14" s="3">
+        <v>31.9128</v>
+      </c>
+      <c r="J14" s="2">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2">
+        <v>18</v>
+      </c>
+      <c r="M14" s="2">
+        <v>7092.7143</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="6">
+        <is>
+          <t>Grand Bus MMC</t>
+        </is>
+      </c>
+      <c r="C15" s="2">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr" s="6">
+        <is>
+          <t>54 118B 148 198</t>
+        </is>
+      </c>
+      <c r="E15" s="3">
+        <v>42.7824</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>1.677</v>
+      </c>
+      <c r="H15" s="2">
+        <v>6</v>
+      </c>
+      <c r="I15" s="3">
+        <v>13.8833</v>
+      </c>
+      <c r="J15" s="2">
+        <v>4</v>
+      </c>
+      <c r="K15" s="2">
+        <v>4</v>
+      </c>
+      <c r="L15" s="2">
+        <v>6</v>
+      </c>
+      <c r="M15" s="2">
+        <v>11057.4286</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="6">
+        <is>
+          <t>Kral Transport MMC</t>
+        </is>
+      </c>
+      <c r="C16" s="2">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr" s="6">
+        <is>
+          <t>39 42 93 132</t>
+        </is>
+      </c>
+      <c r="E16" s="3">
+        <v>50.8253</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>2.1375</v>
+      </c>
+      <c r="H16" s="2">
+        <v>6</v>
+      </c>
+      <c r="I16" s="3">
+        <v>18.006</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2">
+        <v>12</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="6">
+        <is>
+          <t>Transkontrol MMC</t>
+        </is>
+      </c>
+      <c r="C17" s="2">
+        <v>4</v>
+      </c>
+      <c r="D17" t="inlineStr" s="6">
+        <is>
+          <t>113 197 208 209</t>
+        </is>
+      </c>
+      <c r="E17" s="3">
+        <v>41.1927</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>1.9654500000000001</v>
+      </c>
+      <c r="H17" s="2">
+        <v>3</v>
+      </c>
+      <c r="I17" s="3">
+        <v>7.8129</v>
+      </c>
+      <c r="J17" s="2">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2">
+        <v>15</v>
+      </c>
+      <c r="M17" s="2">
+        <v>2054.2857</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="6">
+        <is>
+          <t>ABAS-AĞA BƏDİROV BAHADIR OĞLU</t>
+        </is>
+      </c>
+      <c r="C18" s="2">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr" s="6">
+        <is>
+          <t>536 537</t>
+        </is>
+      </c>
+      <c r="E18" s="3">
+        <v>55.1104</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1.54495</v>
+      </c>
+      <c r="H18" s="2">
+        <v>4</v>
+      </c>
+      <c r="I18" s="3">
+        <v>18.244</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2">
+        <v>13</v>
+      </c>
+      <c r="M18" s="2">
+        <v>5467.5715</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="6">
+        <is>
+          <t>Azlənd Plaza MMC</t>
+        </is>
+      </c>
+      <c r="C19" s="2">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr" s="6">
+        <is>
+          <t>49 161</t>
+        </is>
+      </c>
+      <c r="E19" s="3">
+        <v>37.936</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>2.01735</v>
+      </c>
+      <c r="H19" s="2">
+        <v>3</v>
+      </c>
+      <c r="I19" s="3">
+        <v>8.0232</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0</v>
+      </c>
+      <c r="K19" s="2">
+        <v>0</v>
+      </c>
+      <c r="L19" s="2">
+        <v>20</v>
+      </c>
+      <c r="M19" s="2">
+        <v>2037.0</v>
+      </c>
+      <c r="N19" s="2">
+        <v>19499</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="6">
+        <is>
+          <t>Fidan MMC</t>
+        </is>
+      </c>
+      <c r="C20" s="2">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr" s="6">
+        <is>
+          <t>31 53</t>
+        </is>
+      </c>
+      <c r="E20" s="3">
+        <v>20.8858</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2.15265</v>
+      </c>
+      <c r="H20" s="2">
+        <v>3</v>
+      </c>
+      <c r="I20" s="3">
+        <v>10.3464</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2">
+        <v>0</v>
+      </c>
+      <c r="L20" s="2">
+        <v>4</v>
+      </c>
+      <c r="M20" s="2">
+        <v>5939.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr" s="6">
+        <is>
+          <t>NİCAT FƏRHADOV ZEYNAL OĞLU</t>
+        </is>
+      </c>
+      <c r="C21" s="2">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr" s="6">
+        <is>
+          <t>553 554</t>
+        </is>
+      </c>
+      <c r="E21" s="3">
+        <v>42.0296</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>2.3269</v>
+      </c>
+      <c r="H21" s="2">
+        <v>1</v>
+      </c>
+      <c r="I21" s="3">
+        <v>2.2263</v>
+      </c>
+      <c r="J21" s="2">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2">
+        <v>8</v>
+      </c>
+      <c r="M21" s="2">
+        <v>1632.8572</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr" s="6">
+        <is>
+          <t>RAMİL İSMAYILOV İLHAM OĞLU</t>
+        </is>
+      </c>
+      <c r="C22" s="2">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr" s="6">
+        <is>
+          <t>550 555</t>
+        </is>
+      </c>
+      <c r="E22" s="3">
+        <v>54.713899999999995</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="4">
+        <v>1.4151</v>
+      </c>
+      <c r="H22" s="2">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J22" s="2">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2">
+        <v>0</v>
+      </c>
+      <c r="L22" s="2">
+        <v>9</v>
+      </c>
+      <c r="M22" s="2">
+        <v>4094.1429</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="6">
+        <is>
+          <t>XAN NƏQLİYYAT MMC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="6">
+        <is>
+          <t>Xan Nəqliyyat MMC</t>
+        </is>
+      </c>
+      <c r="C23" s="2">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr" s="6">
+        <is>
+          <t>56 569</t>
+        </is>
+      </c>
+      <c r="E23" s="3">
+        <v>16.2602</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>1.9241000000000001</v>
+      </c>
+      <c r="H23" s="2">
+        <v>2</v>
+      </c>
+      <c r="I23" s="3">
+        <v>6.0242</v>
+      </c>
+      <c r="J23" s="2">
+        <v>0</v>
+      </c>
+      <c r="K23" s="2">
+        <v>0</v>
+      </c>
+      <c r="L23" s="2">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2">
+        <v>18754.4285</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="6">
+        <is>
+          <t>Şidli-A.İ. şirkəti</t>
+        </is>
+      </c>
+      <c r="C24" s="2">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr" s="6">
+        <is>
+          <t>76 78</t>
+        </is>
+      </c>
+      <c r="E24" s="3">
+        <v>15.0866</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>2.77165</v>
+      </c>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="3">
+        <v>1.6114</v>
+      </c>
+      <c r="J24" s="2">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2">
+        <v>15</v>
+      </c>
+      <c r="M24" s="2">
+        <v>2048.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr" s="6">
+        <is>
+          <t>AMAL-D MƏHDUD MƏSULİYYƏTLİ CƏMİYYƏTİ</t>
+        </is>
+      </c>
+      <c r="C25" s="2">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr" s="6">
+        <is>
+          <t>509</t>
+        </is>
+      </c>
+      <c r="E25" s="3">
+        <v>47.5577</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4">
+        <v>1.6152</v>
+      </c>
+      <c r="H25" s="2">
+        <v>2</v>
+      </c>
+      <c r="I25" s="3">
+        <v>14.658</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2">
+        <v>0</v>
+      </c>
+      <c r="L25" s="2">
+        <v>6</v>
+      </c>
+      <c r="M25" s="2">
+        <v>1386.8571</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr" s="6">
+        <is>
+          <t>Bus Service MMC</t>
+        </is>
+      </c>
+      <c r="C26" s="2">
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr" s="6">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="E26" s="3">
+        <v>19.2961</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <v>2.1158</v>
+      </c>
+      <c r="H26" s="2">
+        <v>1</v>
+      </c>
+      <c r="I26" s="3">
+        <v>6.6652</v>
+      </c>
+      <c r="J26" s="2">
+        <v>1</v>
+      </c>
+      <c r="K26" s="2">
+        <v>1</v>
+      </c>
+      <c r="L26" s="2">
+        <v>6</v>
+      </c>
+      <c r="M26" s="2">
+        <v>11721.5714</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr" s="6">
+        <is>
+          <t>ENA Transport MMC</t>
+        </is>
+      </c>
+      <c r="C27" s="2">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr" s="6">
+        <is>
+          <t>567</t>
+        </is>
+      </c>
+      <c r="E27" s="3">
+        <v>18.2631</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4">
+        <v>2.4552</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2">
+        <v>17</v>
+      </c>
+      <c r="M27" s="2">
+        <v>3481.2857</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr" s="6">
+        <is>
+          <t>GÜZDƏK NƏQLİYYAT MMC</t>
+        </is>
+      </c>
+      <c r="C28" s="2">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr" s="6">
+        <is>
+          <t>511</t>
+        </is>
+      </c>
+      <c r="E28" s="3">
+        <v>17.1362</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4">
+        <v>1.2983</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1</v>
+      </c>
+      <c r="I28" s="3">
+        <v>3.567</v>
+      </c>
+      <c r="J28" s="2">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2">
+        <v>1</v>
+      </c>
+      <c r="M28" s="2">
+        <v>7272.4286</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr" s="6">
+        <is>
+          <t>KƏNAN NƏCƏFOV SABİR OĞLU</t>
+        </is>
+      </c>
+      <c r="C29" s="2">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr" s="6">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="E29" s="3">
+        <v>13.062</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1</v>
+      </c>
+      <c r="G29" s="4">
+        <v>1.3372</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J29" s="2">
+        <v>0</v>
+      </c>
+      <c r="K29" s="2">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2">
+        <v>351.5714</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr" s="6">
+        <is>
+          <t>M.S.A.Company MMC</t>
+        </is>
+      </c>
+      <c r="C30" s="2">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr" s="6">
+        <is>
+          <t>525</t>
+        </is>
+      </c>
+      <c r="E30" s="3">
+        <v>18.9184</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="4">
+        <v>2.198</v>
+      </c>
+      <c r="H30" s="2">
+        <v>2</v>
+      </c>
+      <c r="I30" s="3">
+        <v>9.1265</v>
+      </c>
+      <c r="J30" s="2">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2">
+        <v>12</v>
+      </c>
+      <c r="M30" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr" s="6">
+        <is>
+          <t>M.S.S.Company MMC</t>
+        </is>
+      </c>
+      <c r="C31" s="2">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr" s="6">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E31" s="3">
+        <v>13.2209</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1.6463</v>
+      </c>
+      <c r="H31" s="2">
+        <v>2</v>
+      </c>
+      <c r="I31" s="3">
+        <v>6.6751</v>
+      </c>
+      <c r="J31" s="2">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2">
+        <v>12</v>
+      </c>
+      <c r="M31" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr" s="6">
+        <is>
+          <t>Məmmədova Şahnisə Nəsrəddin qızı</t>
+        </is>
+      </c>
+      <c r="C32" s="2">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr" s="6">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="E32" s="3">
+        <v>18.6765</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1.3067</v>
+      </c>
+      <c r="H32" s="2">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J32" s="2">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2">
+        <v>4</v>
+      </c>
+      <c r="M32" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr" s="6">
+        <is>
+          <t>Orucov Malik Ələkbər oğlu</t>
+        </is>
+      </c>
+      <c r="C33" s="2">
+        <v>1</v>
+      </c>
+      <c r="D33" t="inlineStr" s="6">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="E33" s="3">
+        <v>7.8383</v>
+      </c>
+      <c r="F33" s="2">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4">
+        <v>1.8251</v>
+      </c>
+      <c r="H33" s="2">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J33" s="2">
+        <v>0</v>
+      </c>
+      <c r="K33" s="2">
+        <v>0</v>
+      </c>
+      <c r="L33" s="2">
+        <v>3</v>
+      </c>
+      <c r="M33" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr" s="6">
+        <is>
+          <t>Qusar Trans MMC</t>
+        </is>
+      </c>
+      <c r="C34" s="2">
+        <v>1</v>
+      </c>
+      <c r="D34" t="inlineStr" s="6">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="E34" s="3">
+        <v>7.4174</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4">
+        <v>2.1947</v>
+      </c>
+      <c r="H34" s="2">
+        <v>0</v>
+      </c>
+      <c r="I34" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J34" s="2">
+        <v>1</v>
+      </c>
+      <c r="K34" s="2">
+        <v>1</v>
+      </c>
+      <c r="L34" s="2">
+        <v>1</v>
+      </c>
+      <c r="M34" s="2">
+        <v>1518.8571</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr" s="6">
+        <is>
+          <t>SN Cavid MMC</t>
+        </is>
+      </c>
+      <c r="C35" s="2">
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr" s="6">
+        <is>
+          <t>502</t>
+        </is>
+      </c>
+      <c r="E35" s="3">
+        <v>33.8055</v>
+      </c>
+      <c r="F35" s="2">
+        <v>1</v>
+      </c>
+      <c r="G35" s="4">
+        <v>1.0305</v>
+      </c>
+      <c r="H35" s="2">
+        <v>0</v>
+      </c>
+      <c r="I35" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J35" s="2">
+        <v>0</v>
+      </c>
+      <c r="K35" s="2">
+        <v>0</v>
+      </c>
+      <c r="L35" s="2">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2">
+        <v>11419.4286</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr" s="6">
+        <is>
+          <t>STATUS AVTO MMC</t>
+        </is>
+      </c>
+      <c r="C36" s="2">
+        <v>1</v>
+      </c>
+      <c r="D36" t="inlineStr" s="6">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="E36" s="3">
+        <v>35.3186</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4">
+        <v>1.6939</v>
+      </c>
+      <c r="H36" s="2">
+        <v>3</v>
+      </c>
+      <c r="I36" s="3">
+        <v>16.0667</v>
+      </c>
+      <c r="J36" s="2">
+        <v>0</v>
+      </c>
+      <c r="K36" s="2">
+        <v>0</v>
+      </c>
+      <c r="L36" s="2">
+        <v>5</v>
+      </c>
+      <c r="M36" s="2">
+        <v>1046.4286</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr" s="6">
+        <is>
+          <t>SƏMƏD BAYRAMOV ATAKİŞİ OĞLU</t>
+        </is>
+      </c>
+      <c r="C37" s="2">
+        <v>1</v>
+      </c>
+      <c r="D37" t="inlineStr" s="6">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+      <c r="E37" s="3">
+        <v>2.0657</v>
+      </c>
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+      <c r="G37" s="4">
+        <v>1.165</v>
+      </c>
+      <c r="H37" s="2">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J37" s="2">
+        <v>0</v>
+      </c>
+      <c r="K37" s="2">
+        <v>0</v>
+      </c>
+      <c r="L37" s="2">
+        <v>0</v>
+      </c>
+      <c r="M37" s="2">
+        <v>4519.2857</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr" s="6">
+        <is>
+          <t>Vətən firması</t>
+        </is>
+      </c>
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" t="inlineStr" s="6">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E38" s="3">
+        <v>10.6926</v>
+      </c>
+      <c r="F38" s="2">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1.8052</v>
+      </c>
+      <c r="H38" s="2">
+        <v>1</v>
+      </c>
+      <c r="I38" s="3">
+        <v>3.0882</v>
+      </c>
+      <c r="J38" s="2">
+        <v>0</v>
+      </c>
+      <c r="K38" s="2">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2">
+        <v>11</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr" s="6">
+        <is>
+          <t>XƏQANİ ÇIRAQOV MƏMMƏD OĞLU</t>
+        </is>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" t="inlineStr" s="6">
+        <is>
+          <t>521</t>
+        </is>
+      </c>
+      <c r="E39" s="3">
+        <v>14.1311</v>
+      </c>
+      <c r="F39" s="2">
+        <v>1</v>
+      </c>
+      <c r="G39" s="4">
+        <v>1.3062</v>
+      </c>
+      <c r="H39" s="2">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J39" s="2">
+        <v>0</v>
+      </c>
+      <c r="K39" s="2">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2">
+        <v>9</v>
+      </c>
+      <c r="M39" s="2">
+        <v>3982.8571</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr" s="6">
+        <is>
+          <t>Üç qardaş şirkəti</t>
+        </is>
+      </c>
+      <c r="C40" s="2">
+        <v>1</v>
+      </c>
+      <c r="D40" t="inlineStr" s="6">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="E40" s="3">
+        <v>13.2506</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4">
+        <v>2.3767</v>
+      </c>
+      <c r="H40" s="2">
+        <v>3</v>
+      </c>
+      <c r="I40" s="3">
+        <v>8.924</v>
+      </c>
+      <c r="J40" s="2">
+        <v>0</v>
+      </c>
+      <c r="K40" s="2">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2">
+        <v>7</v>
+      </c>
+      <c r="M40" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N40"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>

</xml_diff>

<commit_message>
Redesign research atlas and add recorded coverage sensitivity
</commit_message>
<xml_diff>
--- a/site/checklist.xlsx
+++ b/site/checklist.xlsx
@@ -139,61 +139,68 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="6">
         <is>
-          <t>Data issues: defects found in AYNA's map data that could be fixed at the source.</t>
+          <t>Coverage uses the November 2023 population grid and straight-line distance, not walking access. Finding no uniquely covered population does not establish that riders are unaffected. Geometric detour excess is relative to a straight line, not an achievable saving. Shorter graph paths need checks for legal turns, one-way streets and skipped stops. Shared stops alone do not establish redundant service; close stops are scenario candidates.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="6">
         <is>
-          <t>Detours: stretches where the bus travels at least 2.5 times the straight line between two of its stops, and at least 1.5 km more. Extra minutes are estimates from assumed speeds. The shorter path runs along links buses already drive and is listed when it saves at least 0.5 km.</t>
+          <t>Data issues: defects found in AYNA's map data that could be fixed at the source.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="6">
         <is>
-          <t>Near-duplicate routes: at least 85% of one route's stops are also served by another route (express routes are left out).</t>
+          <t>Detours: stretches where the bus travels at least 2.5 times the straight line between two of its stops, and at least 1.5 km more. Extra minutes are estimates from assumed speeds. The shorter path runs along links buses already drive and is listed when it saves at least 0.5 km.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="6">
         <is>
-          <t>Corridors: stretches of at least 1 km where every link between consecutive stops carries at least 8 routes.</t>
+          <t>Near-duplicate routes: at least 85% of one route's stops are also served by another route (express routes are left out).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="6">
         <is>
-          <t>Close stops: stops less than 250 m along the route from the next stop on every route that uses them, whose removal leaves no gap over 700 m. Terminals and interchange hubs are kept.</t>
+          <t>Corridors: stretches of at least 1 km where every link between consecutive stops carries at least 8 routes.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="6">
         <is>
-          <t>Carriers: the routes each carrier runs and what they measure. AYNA plans the routes, so these figures describe the routes, not how well a carrier runs them. Names that differ only in spelling are counted once.</t>
+          <t>Close stops: stops less than 250 m along the route from the next stop on every route that uses them, whose removal leaves no gap over 700 m. Terminals and interchange hubs are kept.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="6">
         <is>
-          <t>Routes: the measured figures for every route. Residents are counted within 400 m; boardings are published for BakuBus routes only.</t>
+          <t>Carriers: the routes each carrier runs and what they measure. AYNA plans the routes, so these figures describe the routes, not how well a carrier runs them. Names that differ only in spelling are counted once.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="6">
         <is>
-          <t>Page: https://ismatsamadov.github.io/route_efficiency/</t>
+          <t>Routes: the measured figures for every route. Residents are counted within 400 m; boardings are published for BakuBus routes only.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="6">
+        <is>
+          <t>Page: https://ismatsamadov.github.io/route_efficiency/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="6">
         <is>
           <t>Code, data and paper: https://github.com/ismatsamadov/route_efficiency</t>
         </is>
@@ -1135,27 +1142,27 @@
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
-          <t>Residents only this route reaches</t>
+          <t>Population uniquely covered (estimate)</t>
         </is>
       </c>
       <c r="L1" t="inlineStr" s="1">
         <is>
-          <t>Everyone inside has another route</t>
+          <t>No uniquely covered population (grid model)</t>
         </is>
       </c>
       <c r="M1" t="inlineStr" s="1">
         <is>
-          <t>Shorter path, km</t>
+          <t>Graph candidate, km</t>
         </is>
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
-          <t>Saved by it, km</t>
+          <t>Graph distance difference, km</t>
         </is>
       </c>
       <c r="O1" t="inlineStr" s="1">
         <is>
-          <t>Saved by it, minutes (estimate)</t>
+          <t>Modelled time difference, minutes</t>
         </is>
       </c>
       <c r="P1" t="inlineStr" s="1">

</xml_diff>